<commit_message>
Rounding is one per study: a study sheet instead of tables$rounding
A study that rounds two tables differently is inconsistent by
construction, so the rounding family moves off the per-report `tables`
sheet onto a new `study` sheet (key / value, no output_id).  A `rounding`
column on `tables` is refused, naming the `study` sheet.  Example
workbooks rebuilt; spec == code still holds for all ten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="_README" sheetId="1" r:id="rId1"/>
-    <sheet name="tables" sheetId="2" r:id="rId2"/>
-    <sheet name="variables" sheetId="3" r:id="rId3"/>
-    <sheet name="cells" sheetId="4" r:id="rId4"/>
-    <sheet name="about" sheetId="5" r:id="rId5"/>
+    <sheet name="study" sheetId="2" r:id="rId2"/>
+    <sheet name="tables" sheetId="3" r:id="rId3"/>
+    <sheet name="variables" sheetId="4" r:id="rId4"/>
+    <sheet name="cells" sheetId="5" r:id="rId5"/>
+    <sheet name="about" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -355,7 +356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -405,7 +406,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>すべてのシートの先頭列。空欄 = 試験全体のデフォルト。帳票名を書いた行は、同じキーのデフォルト行を置き換える。</t>
+          <t>tables / variables / cells の先頭列。空欄 = 試験全体のデフォルト。帳票名を書いた行は、同じキーのデフォルト行を置き換える。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -456,34 +457,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tables</t>
+          <t>study</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1 行 = 1 帳票。役割と表全体のオプション。コードで同じ引数を書けばそちらが勝つ。</t>
+          <t>試験で 1 つに決まる事実。key / value の 2 列、1 行 = 1 項目。output_id は無い（帳票ごとに変えられない）。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tables</t>
+          <t>study</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>cols</t>
+          <t>rounding</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>横に展開するキー。外側から順に。</t>
+          <t>丸め方。r（偶数丸め）/ sas（四捨五入）。試験内のすべての帳票に効く。空欄 = options(rtfreporter.rounding)。</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TR01AG1 | SEROSTAT</t>
+          <t>sas</t>
         </is>
       </c>
     </row>
@@ -493,19 +494,9 @@
           <t>tables</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>rows</t>
-        </is>
-      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>縦のキー。name = 列名 で列名を付け替え。引用符で囲んだ値は固定の見出し。</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>group1 = AEBODSYS | grp = "Worst Post-Baseline Values"</t>
+          <t>1 行 = 1 帳票。役割と表全体のオプション。コードで同じ引数を書けばそちらが勝つ。</t>
         </is>
       </c>
     </row>
@@ -517,17 +508,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>cols</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>行ラベルの元。空欄 = .label。NA = 行の区別にだけ使って列は出さない。NULL = 使わない。</t>
+          <t>横に展開するキー。外側から順に。</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>label = AEDECOD</t>
+          <t>TR01AG1 | SEROSTAT</t>
         </is>
       </c>
     </row>
@@ -539,17 +530,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>stats</t>
+          <t>rows</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>cells（テンプレートでセルを作る）/ rows（統計量ごとに 1 行、生の値）。</t>
+          <t>縦のキー。name = 列名 で列名を付け替え。引用符で囲んだ値は固定の見出し。</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>rows</t>
+          <t>group1 = AEBODSYS | grp = "Worst Post-Baseline Values"</t>
         </is>
       </c>
     </row>
@@ -561,17 +552,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>stats = rows のときの値。stat（数値）/ stat_fmt（cards 整形済み文字列）。</t>
+          <t>行ラベルの元。空欄 = .label。NA = 行の区別にだけ使って列は出さない。NULL = 使わない。</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>stat</t>
+          <t>label = AEDECOD</t>
         </is>
       </c>
     </row>
@@ -583,17 +574,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>sep</t>
+          <t>stats</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>cols が複数のとき列名をつなぐ文字。既定は ____。</t>
+          <t>cells（テンプレートでセルを作る）/ rows（統計量ごとに 1 行、生の値）。</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>_</t>
+          <t>rows</t>
         </is>
       </c>
     </row>
@@ -605,17 +596,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>sort</t>
+          <t>value</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TRUE / FALSE / 並べ替えキーの列挙。</t>
+          <t>stats = rows のときの値。stat（数値）/ stat_fmt（cards 整形済み文字列）。</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>.overall | group1 | .depth | -n | label</t>
+          <t>stat</t>
         </is>
       </c>
     </row>
@@ -627,17 +618,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>sort_stat</t>
+          <t>sep</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>列方向に合計して .sort_stat 列にする統計量名。</t>
+          <t>cols が複数のとき列名をつなぐ文字。既定は ____。</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>_</t>
         </is>
       </c>
     </row>
@@ -649,17 +640,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>na</t>
+          <t>sort</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>どのテンプレートも埋められなかったセルの値。</t>
+          <t>TRUE / FALSE / 並べ替えキーの列挙。</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>.overall | group1 | .depth | -n | label</t>
         </is>
       </c>
     </row>
@@ -671,29 +662,39 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>rounding</t>
+          <t>sort_stat</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>丸め方。r（偶数丸め）/ sas（四捨五入）。空欄 = options(rtfreporter.rounding)。</t>
+          <t>列方向に合計して .sort_stat 列にする統計量名。</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>sas</t>
+          <t>n</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>variables</t>
+          <t>tables</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>na</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1 行 = 1 変数。解析変数だけでなく列キーやラベル列の名前も書ける。</t>
+          <t>どのテンプレートも埋められなかったセルの値。</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -703,19 +704,9 @@
           <t>variables</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>変数名（解析変数・列キー・ラベル列名）。</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>AGEGR1</t>
+          <t>1 行 = 1 変数。解析変数だけでなく列キーやラベル列の名前も書ける。</t>
         </is>
       </c>
     </row>
@@ -727,17 +718,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>変数名の代わりに表示する文字。</t>
+          <t>変数名（解析変数・列キー・ラベル列名）。</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Age (years)</t>
+          <t>AGEGR1</t>
         </is>
       </c>
     </row>
@@ -749,17 +740,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>order</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>変数の出現順（数値）。</t>
+          <t>変数名の代わりに表示する文字。</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Age (years)</t>
         </is>
       </c>
     </row>
@@ -771,29 +762,39 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>levels</t>
+          <t>order</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>値の並び順。</t>
+          <t>変数の出現順（数値）。</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Grade 0 | Grade 1 | Total</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cells</t>
+          <t>variables</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>levels</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1 行 = セルの 1 行分のテンプレート。同じ variable / context / row の行は上から順に試す連鎖になる。</t>
+          <t>値の並び順。</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Grade 0 | Grade 1 | Total</t>
         </is>
       </c>
     </row>
@@ -803,19 +804,9 @@
           <t>cells</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>対象。変数名、または continuous / categorical、空欄 = すべてのデフォルト。</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>continuous</t>
+          <t>1 行 = セルの 1 行分のテンプレート。同じ variable / context / row の行は上から順に試す連鎖になる。</t>
         </is>
       </c>
     </row>
@@ -827,17 +818,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ARD の context で絞るとき（同じ変数を 2 通りに集計した場合など）。</t>
+          <t>対象。変数名、または continuous / categorical、空欄 = すべてのデフォルト。</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
@@ -849,17 +840,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>row</t>
+          <t>context</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>行ラベル。空欄 = 水準ごとに 1 行（ラベルは水準名）。</t>
+          <t>ARD の context で絞るとき（同じ変数を 2 通りに集計した場合など）。</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mean (SD)</t>
+          <t>summary</t>
         </is>
       </c>
     </row>
@@ -871,17 +862,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>when</t>
+          <t>row</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>条件（R の式）。成り立つときだけこの行を使う。空欄 = 無条件。</t>
+          <t>行ラベル。空欄 = 水準ごとに 1 行（ラベルは水準名）。</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>n == 0</t>
+          <t>Mean (SD)</t>
         </is>
       </c>
     </row>
@@ -893,17 +884,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>when</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>セルの書き方。{統計量:書式} を埋め込む。</t>
+          <t>条件（R の式）。成り立つときだけこの行を使う。空欄 = 無条件。</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>{mean} ({sd})</t>
+          <t>n == 0</t>
         </is>
       </c>
     </row>
@@ -915,17 +906,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>digits</t>
+          <t>template</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>書式のないトークンの小数桁。カンマ区切りでトークンごと。</t>
+          <t>セルの書き方。{統計量:書式} を埋め込む。</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2,3</t>
+          <t>{mean} ({sd})</t>
         </is>
       </c>
     </row>
@@ -937,49 +928,71 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>signif</t>
+          <t>digits</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>有効桁（digits より優先）。</t>
+          <t>書式のないトークンの小数桁。カンマ区切りでトークンごと。</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2,3</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>about</t>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>signif</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
+          <t>有効桁（digits より優先）。</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>spec_version = 1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>about</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>spec_version = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>(予約)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>次の版で読む予定のシート名。今は置いても読まれず、その旨のメッセージが出る。</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>titles / footnotes / page / header / footer / columns / layout / style</t>
         </is>
@@ -992,105 +1005,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>output_id</t>
+          <t>key</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>cols</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>rows</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>stats</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
           <t>value</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>sep</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>sort</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>sort_stat</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>na</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>rounding</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>rounding</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TR01AG1 | SEROSTAT</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>group1 = AEBODSYS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>label = AEDECOD</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>.overall | group1 | .depth | -n | label</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
           <t>sas</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>TEAE by SOC / PT, frequency descending</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1039,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1112,22 +1050,52 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>cols</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>order</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>levels</t>
+          <t>stats</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>sep</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>sort</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>sort_stat</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
         </is>
       </c>
     </row>
@@ -1139,29 +1107,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TR01AG1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Placebo | Xanomeline Low Dose | Xanomeline High Dose</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AE</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SEROSTAT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Positive | Negative</t>
+          <t>TR01AG1 | SEROSTAT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>group1 = AEBODSYS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>label = AEDECOD</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>.overall | group1 | .depth | -n | label</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>TEAE by SOC / PT, frequency descending</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1138,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1188,32 +1154,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>label</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>row</t>
+          <t>order</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>when</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>digits</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>signif</t>
+          <t>levels</t>
         </is>
       </c>
     </row>
@@ -1223,9 +1174,31 @@
           <t>AE</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>{n:.0f} ({p:.1f%})</t>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TR01AG1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Placebo | Xanomeline Low Dose | Xanomeline High Dose</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SEROSTAT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Positive | Negative</t>
         </is>
       </c>
     </row>
@@ -1236,6 +1209,70 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>variable</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>when</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>digits</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>signif</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>{n:.0f} ({p:.1f%})</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
A workbook goes to rtftable pages: layout / columns / style sheets
Three sheets carry the table half -- layout (pages_*, group_*, blank_*,
stub_*, colpages_*, each prefix its plan verb), columns (by name, with
.values for every spread column: width, row_title, decimal_split, hide)
and style -- and a cells row with no template is a stats = rows
statistic's format.  Values are typed and checked where written.

One entry point: rtf_plan(data, spec = ) reads the workbook as the plan's
first layers, so a verb written after it still wins.  ard_spread(spec = )
and ard_template(spec = ) are withdrawn.  Fixes a `$` partial match that
turned group_collapse into the grouping column.

Examples rebuilt; each workbook now also gives the identical rtftable
pages to its report's plan code (10/10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -12,7 +12,10 @@
     <sheet name="tables" sheetId="3" r:id="rId3"/>
     <sheet name="variables" sheetId="4" r:id="rId4"/>
     <sheet name="cells" sheetId="5" r:id="rId5"/>
-    <sheet name="about" sheetId="6" r:id="rId6"/>
+    <sheet name="layout" sheetId="6" r:id="rId6"/>
+    <sheet name="columns" sheetId="7" r:id="rId7"/>
+    <sheet name="style" sheetId="8" r:id="rId8"/>
+    <sheet name="about" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -356,7 +359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -389,7 +392,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter の ARD 定義ファイル（spec_version 1）。ard_spread(spec = read_ard_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
+          <t>rtfreporter の ARD 定義ファイル（spec_version 1）。rtf_plan(data; spec = read_ard_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
         </is>
       </c>
     </row>
@@ -967,34 +970,356 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>about</t>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>（template 空欄の行）</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
+          <t>stats = rows の帳票だけ：統計量ごとの表示桁。row = 統計量名（ラベル列の値）、digits / signif を書く（fmt_numeric と同じ）。variable / context は空欄。</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>spec_version = 1</t>
+          <t>row = Mean / signif = 4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>(全体)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>（読み方）</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ここまでの 4 シートで table data.frame、以下の 3 シートで rtftable のページまで。rtf_plan(data; spec = read_ard_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1 行 = 1 帳票。ページ・グループ・空行・スタブ。列名の接頭辞が対応する plan_*() を表す。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>pages_max_rows / pages_split / pages_by / pages_min_group_rows / pages_cont_label</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>26 / group_force / " (Cont.)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>group_col / group_mode / group_collapse</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>value / 1 | 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>group_page / group_show</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>group_page = TRUE で group_col の値ごとに改ページ（plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>TRUE / FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>blank_where / blank_first / blank_last / blank_counted</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>plan_blanks() の where / first / last / counted。</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>between_groups / TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>stub_vars / stub_into / stub_indent / stub_summary / stub_before</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>plan_stub() の vars / into / indent / group_summary / before。</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>row_label / TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>colpages_every / colpages_at / colpages_carry / colpages_order</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>16 | 29 / 1 | 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1 行 = 印字される列 1 つ。列は名前で指定（畳んだスタブは stub_into の名前）。.values = 展開された値の列すべて。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>列名、または .values。</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>相対幅。幅を書くなら印字される全列に必要（.values でまとめて指定できる）。</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>row_title</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>TRUE で行見出しの列。</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>decimal_split</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>TRUE で小数点を揃える（set_decimal_split）。</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>hide</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TRUE で処理には使うが印字しない。</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>style</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1 行 = 1 帳票。border / align_count_pct / auto_width / row_height_twips / header_row_height_twips / blank_row_height_twips / font / font_size_half_points / table_align / cell_valign（rtftable と同じ引数）。</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>align_count_pct = TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>about</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>spec_version = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>(予約)</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>次の版で読む予定のシート名。今は置いても読まれず、その旨のメッセージが出る。</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>titles / footnotes / page / header / footer / columns / layout / style</t>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>titles / footnotes / page / header / footer / cell_styles</t>
         </is>
       </c>
     </row>
@@ -1273,6 +1598,345 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:X2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>pages_max_rows</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pages_split</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>pages_by</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>pages_min_group_rows</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>pages_cont_label</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>group_col</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>group_mode</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>group_collapse</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>group_page</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>group_show</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>blank_where</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>blank_first</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>blank_last</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>blank_counted</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>stub_vars</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>stub_into</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>stub_indent</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>stub_summary</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>stub_before</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_every</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_at</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_carry</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>group_force</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>between_groups</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>row_title</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>decimal_split</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>hide</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>output_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>border</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>align_count_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>auto_width</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>row_height_twips</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>header_row_height_twips</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>blank_row_height_twips</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>font</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>font_size_half_points</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>table_align</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>cell_valign</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
The column header is a workbook sheet: col_header
One row per header cell (line, cols, span, text, align, bold, borders).
cols takes names, .values, positions and KEY = value; span makes one
cell, one per column, or one spanner per value of a column key.  The
plan_col_header() tokens work, and {n} is read from the ARD whenever a
text uses it.  It resolves on the finished page to the rtf_col_header()
a hand-written header would be.

Example workbooks carry their headers; each gives the identical pages,
header included, to its report's plan code (10/10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -15,7 +15,8 @@
     <sheet name="layout" sheetId="6" r:id="rId6"/>
     <sheet name="columns" sheetId="7" r:id="rId7"/>
     <sheet name="style" sheetId="8" r:id="rId8"/>
-    <sheet name="about" sheetId="9" r:id="rId9"/>
+    <sheet name="col_header" sheetId="9" r:id="rId9"/>
+    <sheet name="about" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -359,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1002,7 +1003,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ここまでの 4 シートで table data.frame、以下の 3 シートで rtftable のページまで。rtf_plan(data; spec = read_ard_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。rtf_plan(data; spec = read_ard_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
         </is>
       </c>
     </row>
@@ -1292,34 +1293,190 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>about</t>
+          <t>col_header</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>spec_version = 1</t>
+          <t>1 行 = 列ヘッダーのセル 1 つ。帳票の行があればデフォルトのヘッダーを丸ごと置き換える。</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>col_header</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ヘッダーの行番号（1 = 一番上）。</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>col_header</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>cols</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>セルが乗る列。列名 / .values（値の列すべて）/ 位置（3、3:31、3:last）/ KEY = 値（そのキーがその値の列）を | 区切りで。</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>.values / grp1 | grp2 / variable = n</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>col_header</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>空欄 = cols 全体で 1 セル。each = 列ごとに 1 セル。キー名 = そのキーの値ごとに 1 セル（群のスパナー）。</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TR01AG1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>col_header</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>表示文字。改行は Alt+Enter か \n。{col} {col1} {col2} {n} {n:sum} が使える。{n} を使うと N は ARD から取る。先頭の空白は引用符で囲む。</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>{col1}\n(N={n:sum})</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>col_header</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>align / bold / border_top / border_bottom</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>col_cell() / rtf_border() と同じ（single / none など）。</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>about</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>spec_version = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>(予約)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>次の版で読む予定のシート名。今は置いても読まれず、その旨のメッセージが出る。</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>titles / footnotes / page / header / footer / cell_styles</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>spec_version</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1937,30 +2094,199 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>output_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cols</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>align</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>border_top</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>border_bottom</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>spec_version</t>
+          <t>AE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TR01AG1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{col1}
+(N={n:sum})
+ n (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TR01AG1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>System Organ Class
+   Preferred Term</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{col2}
+(N={n})</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Header {n}: choose the page's population or the analysis set
On pages split by a group value a header's N can be the page's own
population (the subjects with that lab test: ARD rows carrying the page
key) or the analysis set (rows without it).  plan_col_header(n = "page")
or n = "table" says which; n = list(n = "page", N = "table") gives both
as {n} and {N}; the tables sheet takes the same as `header_n`.  Both
must be in the ARD -- neither is filled in from outside it.  n = TRUE
reads the page's and warns when the ARD states both and they differ.
One warning per missing number, not one per page.

The bundled workbooks gain the empty `header_n` column; their _README
sheet describes it.

Refs #482

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/ard-spec/AE.xlsx
+++ b/inst/extdata/ard-spec/AE.xlsx
@@ -366,7 +366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -711,12 +711,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>variables</t>
+          <t>tables</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>header_n</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1 行 = 1 変数。解析変数だけでなく列キーやラベル列の名前も書ける。</t>
+          <t>ページ（検査項目など）で分けた表のヘッダー {n} がどの母集団か。page = そのページの母集団（その検査を受けた人）/ table = 解析対象集団（ページキーを持たない ARD 行）。両方なら n = page | N = table で {n} と {N}。空欄 = page（両方あって食い違えば警告）。どちらも ARD に入れておくこと。</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>n = page | N = table</t>
         </is>
       </c>
     </row>
@@ -726,19 +736,9 @@
           <t>variables</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>変数名（解析変数・列キー・ラベル列名）。</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>AGEGR1</t>
+          <t>1 行 = 1 変数。解析変数だけでなく列キーやラベル列の名前も書ける。</t>
         </is>
       </c>
     </row>
@@ -750,17 +750,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>変数名の代わりに表示する文字。</t>
+          <t>変数名（解析変数・列キー・ラベル列名）。</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Age (years)</t>
+          <t>AGEGR1</t>
         </is>
       </c>
     </row>
@@ -772,17 +772,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>order</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>変数の出現順（数値）。</t>
+          <t>変数名の代わりに表示する文字。</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Age (years)</t>
         </is>
       </c>
     </row>
@@ -794,29 +794,39 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>levels</t>
+          <t>order</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>値の並び順。</t>
+          <t>変数の出現順（数値）。</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Grade 0 | Grade 1 | Total</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cells</t>
+          <t>variables</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>levels</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1 行 = セルの 1 行分のテンプレート。同じ variable / context / row の行は上から順に試す連鎖になる。</t>
+          <t>値の並び順。</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Grade 0 | Grade 1 | Total</t>
         </is>
       </c>
     </row>
@@ -826,19 +836,9 @@
           <t>cells</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>対象。変数名、または continuous / categorical、空欄 = すべてのデフォルト。</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>continuous</t>
+          <t>1 行 = セルの 1 行分のテンプレート。同じ variable / context / row の行は上から順に試す連鎖になる。</t>
         </is>
       </c>
     </row>
@@ -850,17 +850,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ARD の context で絞るとき（同じ変数を 2 通りに集計した場合など）。</t>
+          <t>対象。変数名、または continuous / categorical、空欄 = すべてのデフォルト。</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
@@ -872,17 +872,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>row</t>
+          <t>context</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>行ラベル。空欄 = 水準ごとに 1 行（ラベルは水準名）。</t>
+          <t>ARD の context で絞るとき（同じ変数を 2 通りに集計した場合など）。</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mean (SD)</t>
+          <t>summary</t>
         </is>
       </c>
     </row>
@@ -894,17 +894,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>when</t>
+          <t>row</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>条件（R の式）。成り立つときだけこの行を使う。空欄 = 無条件。</t>
+          <t>行ラベル。空欄 = 水準ごとに 1 行（ラベルは水準名）。</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>n == 0</t>
+          <t>Mean (SD)</t>
         </is>
       </c>
     </row>
@@ -916,17 +916,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>template</t>
+          <t>when</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>セルの書き方。{統計量:書式} を埋め込む。</t>
+          <t>条件（R の式）。成り立つときだけこの行を使う。空欄 = 無条件。</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>{mean} ({sd})</t>
+          <t>n == 0</t>
         </is>
       </c>
     </row>
@@ -938,17 +938,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>digits</t>
+          <t>template</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>書式のないトークンの小数桁。カンマ区切りでトークンごと。</t>
+          <t>セルの書き方。{統計量:書式} を埋め込む。</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2,3</t>
+          <t>{mean} ({sd})</t>
         </is>
       </c>
     </row>
@@ -960,17 +960,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>signif</t>
+          <t>digits</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>有効桁（digits より優先）。</t>
+          <t>書式のないトークンの小数桁。カンマ区切りでトークンごと。</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2,3</t>
         </is>
       </c>
     </row>
@@ -982,46 +982,56 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>（template 空欄の行）</t>
+          <t>signif</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>stats = rows の帳票だけ：統計量ごとの表示桁。row = 統計量名（ラベル列の値）、digits / signif を書く（fmt_numeric と同じ）。variable / context は空欄。</t>
+          <t>有効桁（digits より優先）。</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>row = Mean / signif = 4</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>(全体)</t>
+          <t>cells</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>（読み方）</t>
+          <t>（template 空欄の行）</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+          <t>stats = rows の帳票だけ：統計量ごとの表示桁。row = 統計量名（ラベル列の値）、digits / signif を書く（fmt_numeric と同じ）。variable / context は空欄。</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>row = Mean / signif = 4</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>(全体)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>（読み方）</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1 行 = 1 帳票。ページ・グループ・空行・スタブ。列名の接頭辞が対応する plan_*() を表す。</t>
+          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
         </is>
       </c>
     </row>
@@ -1031,19 +1041,9 @@
           <t>layout</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>pages_max_rows / pages_split / pages_by / pages_min_group_rows / pages_cont_label</t>
-        </is>
-      </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>26 / group_force / " (Cont.)"</t>
+          <t>1 行 = 1 帳票。ページ・グループ・空行・スタブ。列名の接頭辞が対応する plan_*() を表す。</t>
         </is>
       </c>
     </row>
@@ -1055,17 +1055,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>group_col / group_mode / group_collapse</t>
+          <t>pages_max_rows / pages_split / pages_by / pages_min_group_rows / pages_cont_label</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
+          <t>plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>value / 1 | 2</t>
+          <t>26 / group_force / " (Cont.)"</t>
         </is>
       </c>
     </row>
@@ -1077,17 +1077,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>group_page / group_show</t>
+          <t>group_col / group_mode / group_collapse</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>group_page = TRUE で group_col の値ごとに改ページ（plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
+          <t>plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>TRUE / FALSE</t>
+          <t>value / 1 | 2</t>
         </is>
       </c>
     </row>
@@ -1099,17 +1099,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>blank_where / blank_first / blank_last / blank_counted</t>
+          <t>group_page / group_show</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>plan_blanks() の where / first / last / counted。</t>
+          <t>group_page = TRUE で group_col の値ごとに改ページ（plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>between_groups / TRUE</t>
+          <t>TRUE / FALSE</t>
         </is>
       </c>
     </row>
@@ -1121,17 +1121,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>stub_vars / stub_into / stub_indent / stub_summary / stub_before</t>
+          <t>blank_where / blank_first / blank_last / blank_counted</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>plan_stub() の vars / into / indent / group_summary / before。</t>
+          <t>plan_blanks() の where / first / last / counted。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>row_label / TRUE</t>
+          <t>between_groups / TRUE</t>
         </is>
       </c>
     </row>
@@ -1143,29 +1143,39 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>colpages_every / colpages_at / colpages_carry / colpages_order</t>
+          <t>stub_vars / stub_into / stub_indent / stub_summary / stub_before</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
+          <t>plan_stub() の vars / into / indent / group_summary / before。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>16 | 29 / 1 | 2</t>
+          <t>row_label / TRUE</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>columns</t>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>colpages_every / colpages_at / colpages_carry / colpages_order</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1 行 = 印字される列 1 つ。列は名前で指定（畳んだスタブは stub_into の名前）。.values = 展開された値の列すべて。</t>
+          <t>plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>16 | 29 / 1 | 2</t>
         </is>
       </c>
     </row>
@@ -1175,19 +1185,9 @@
           <t>columns</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>列名、または .values。</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>row_label</t>
+          <t>1 行 = 印字される列 1 つ。列は名前で指定（畳んだスタブは stub_into の名前）。.values = 展開された値の列すべて。</t>
         </is>
       </c>
     </row>
@@ -1199,17 +1199,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>width</t>
+          <t>column</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>相対幅。幅を書くなら印字される全列に必要（.values でまとめて指定できる）。</t>
+          <t>列名、または .values。</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>row_label</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1221,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>row_title</t>
+          <t>width</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TRUE で行見出しの列。</t>
+          <t>相対幅。幅を書くなら印字される全列に必要（.values でまとめて指定できる）。</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1243,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>decimal_split</t>
+          <t>row_title</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TRUE で小数点を揃える（set_decimal_split）。</t>
+          <t>TRUE で行見出しの列。</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>hide</t>
+          <t>decimal_split</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TRUE で処理には使うが印字しない。</t>
+          <t>TRUE で小数点を揃える（set_decimal_split）。</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1282,29 +1282,39 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>style</t>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>hide</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1 行 = 1 帳票。border / align_count_pct / auto_width / row_height_twips / header_row_height_twips / blank_row_height_twips / font / font_size_half_points / table_align / cell_valign（rtftable と同じ引数）。</t>
+          <t>TRUE で処理には使うが印字しない。</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>align_count_pct = TRUE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>col_header</t>
+          <t>style</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1 行 = 列ヘッダーのセル 1 つ。帳票の行があればデフォルトのヘッダーを丸ごと置き換える。</t>
+          <t>1 行 = 1 帳票。border / align_count_pct / auto_width / row_height_twips / header_row_height_twips / blank_row_height_twips / font / font_size_half_points / table_align / cell_valign（rtftable と同じ引数）。</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>align_count_pct = TRUE</t>
         </is>
       </c>
     </row>
@@ -1314,19 +1324,9 @@
           <t>col_header</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>line</t>
-        </is>
-      </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ヘッダーの行番号（1 = 一番上）。</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>1</t>
+          <t>1 行 = 列ヘッダーのセル 1 つ。帳票の行があればデフォルトのヘッダーを丸ごと置き換える。</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>cols</t>
+          <t>line</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>セルが乗る列。列名 / .values（値の列すべて）/ 位置（3、3:31、3:last）/ KEY = 値（そのキーがその値の列）を | 区切りで。</t>
+          <t>ヘッダーの行番号（1 = 一番上）。</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>.values / grp1 | grp2 / variable = n</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1360,17 +1360,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>span</t>
+          <t>cols</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>空欄 = cols 全体で 1 セル。each = 列ごとに 1 セル。キー名 = そのキーの値ごとに 1 セル（群のスパナー）。</t>
+          <t>セルが乗る列。列名 / .values（値の列すべて）/ 位置（3、3:31、3:last）/ KEY = 値（そのキーがその値の列）を | 区切りで。</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>TR01AG1</t>
+          <t>.values / grp1 | grp2 / variable = n</t>
         </is>
       </c>
     </row>
@@ -1382,17 +1382,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>span</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>表示文字。改行は Alt+Enter か \n。{col} {col1} {col2} {n} {n:sum} が使える。{n} を使うと N は ARD から取る。先頭の空白は引用符で囲む。</t>
+          <t>空欄 = cols 全体で 1 セル。each = 列ごとに 1 セル。キー名 = そのキーの値ごとに 1 セル（群のスパナー）。</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>{col1}\n(N={n:sum})</t>
+          <t>TR01AG1</t>
         </is>
       </c>
     </row>
@@ -1404,185 +1404,207 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>align / bold / border_top / border_bottom</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>col_cell() / rtf_border() と同じ（single / none など）。</t>
+          <t>表示文字。改行は Alt+Enter か \n。{col} {col1} {col2} {n} {n:sum} が使える。{n} を使うと N は ARD から取る。先頭の空白は引用符で囲む。</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>{col1}\n(N={n:sum})</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>(帳票全体)</t>
+          <t>col_header</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>（読み方）</t>
+          <t>align / bold / border_top / border_bottom</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>以下は表の周りの定義。read_report_spec(c(report.xlsx; tables.xlsx); output_id = ) で 1 冊でも分冊でも読める。同じシートに行があるのは 1 冊だけにする（空のシートと study は重なってよい）。rtf_report(spec; plan) で rtf_document、report_path(spec) で出力先。</t>
+          <t>col_cell() / rtf_border() と同じ（single / none など）。</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>single</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>(帳票全体)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>output_path / program_dir</t>
+          <t>（読み方）</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>出力先フォルダ / プログラムのフォルダ（{PROGRAM} に使う）。</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>../tables / C:\study\tfl</t>
+          <t>以下は表の周りの定義。read_report_spec(c(report.xlsx; tables.xlsx); output_id = ) で 1 冊でも分冊でも読める。同じシートに行があるのは 1 冊だけにする（空のシートと study は重なってよい）。rtf_report(spec; plan) で rtf_document、report_path(spec) で出力先。</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>report</t>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>output_path / program_dir</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>1 行 = 1 帳票（空欄 = 試験の既定）。type（table / listing / figure）、file（既定 {output_id}.rtf）、program（既定 {output_id}）、auto_section、section_align、auto_title、title_align、table_font_size / title_font_size / footnote_font_size（半ポイント）、page_header / page_footer（FALSE でその帳票だけ付けない）。</t>
+          <t>出力先フォルダ / プログラムのフォルダ（{PROGRAM} に使う）。</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>auto_section = TRUE</t>
+          <t>../tables / C:\study\tfl</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>page</t>
+          <t>report</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1 行 = 1 帳票（空欄 = 試験の既定）。paper_size、orientation、width_in、height_in、margin_*_in、header_dist_in、footer_dist_in、font_size_half_points、title_format、footnote_format、title_width、footnote_width、markup。</t>
+          <t>1 行 = 1 帳票（空欄 = 試験の既定）。type（table / listing / figure）、file（既定 {output_id}.rtf）、program（既定 {output_id}）、auto_section、section_align、auto_title、title_align、table_font_size / title_font_size / footnote_font_size（半ポイント）、page_header / page_footer（FALSE でその帳票だけ付けない）。</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>A4 / landscape / 0.5</t>
+          <t>auto_section = TRUE</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>header</t>
+          <t>page</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ページヘッダーの 1 行 = 1 行。line がキー：試験共通を空欄 output_id の 1・2 行目に、帳票のタイトルをその帳票の 3 行目以降に。left / center / right。文字のない行は空行。</t>
+          <t>1 行 = 1 帳票（空欄 = 試験の既定）。paper_size、orientation、width_in、height_in、margin_*_in、header_dist_in、footer_dist_in、font_size_half_points、title_format、footnote_format、title_width、footnote_width、markup。</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>1 / TAKEDA / / Interim Analysis</t>
+          <t>A4 / landscape / 0.5</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>footer</t>
+          <t>header</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ページフッターの 1 行 = 1 行。帳票の脚注を 1 行目から、実行情報を空欄 output_id の 99 行目に 1 回だけ書けば全帳票の最後に付く。</t>
+          <t>ページヘッダーの 1 行 = 1 行。line がキー：試験共通を空欄 output_id の 1・2 行目に、帳票のタイトルをその帳票の 3 行目以降に。left / center / right。文字のない行は空行。</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>99 / {PROGRAM}       Generated on: {DATETIME}</t>
+          <t>1 / TAKEDA / / Interim Analysis</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>titles / footnotes</t>
+          <t>footer</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>本文（表の上 / 下）のタイトル・脚注。書き方は header と同じ。</t>
+          <t>ページフッターの 1 行 = 1 行。帳票の脚注を 1 行目から、実行情報を空欄 output_id の 99 行目に 1 回だけ書けば全帳票の最後に付く。</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>1 / CV = Coefficient of variation</t>
+          <t>99 / {PROGRAM}       Generated on: {DATETIME}</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>（差し込み記号）</t>
+          <t>titles / footnotes</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>{PAGE} {TOTAL_PAGES} {AUTO_PAGE} {AUTO_TOTAL_PAGES}（ページ番号）、{PROGRAM} {PROGRAM_NAME} {PROGRAM_DIR}（プログラム）、{DATETIME} {DATETIME:%Y-%m-%d}（作成日時）。</t>
+          <t>本文（表の上 / 下）のタイトル・脚注。書き方は header と同じ。</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1 / CV = Coefficient of variation</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>about</t>
+          <t>（差し込み記号）</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>spec_version = 1</t>
+          <t>{PAGE} {TOTAL_PAGES} {AUTO_PAGE} {AUTO_TOTAL_PAGES}（ページ番号）、{PROGRAM} {PROGRAM_NAME} {PROGRAM_DIR}（プログラム）、{DATETIME} {DATETIME:%Y-%m-%d}（作成日時）。</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>about</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>key / value。spec_version を記録（新しい版のファイルを古いパッケージで読むとエラー）。</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>spec_version = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>(予約)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>次の版で読む予定のシート名。今は置いても読まれず、その旨のメッセージが出る。</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>cell_styles / listing / listing_cols / figures</t>
         </is>
@@ -1999,7 +2021,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2055,6 +2077,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>header_n</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -2085,7 +2112,7 @@
           <t>.overall | group1 | .depth | -n | label</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>TEAE by SOC / PT, frequency descending</t>
         </is>

</xml_diff>